<commit_message>
Rhéo mayo dans excel
</commit_message>
<xml_diff>
--- a/Experiences/Mesures mayonnaise.xlsx
+++ b/Experiences/Mesures mayonnaise.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Mines IC\TR Fluide\VS\Experiences\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC80C580-B8C1-4651-B134-05D13635F4CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10602154-A4DE-4D03-AF1B-36EDA3C5D8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{55767A0E-F7C5-4F3D-85D9-C64A23758580}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{55767A0E-F7C5-4F3D-85D9-C64A23758580}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -90,10 +90,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,26 +452,26 @@
       <c r="B2" s="1">
         <v>5.0121400000000003E-2</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2">
         <v>10.7</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2">
         <v>18.899999999999999</v>
       </c>
       <c r="E2" s="1">
         <v>1009</v>
       </c>
       <c r="F2" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G2" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H2" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I2" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J2" s="1">
         <v>9.81</v>
@@ -485,26 +484,26 @@
       <c r="B3" s="1">
         <v>5.0121400000000003E-2</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3">
         <v>10.8</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3">
         <v>19</v>
       </c>
       <c r="E3" s="1">
         <v>1009</v>
       </c>
       <c r="F3" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G3" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H3" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I3" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J3" s="1">
         <v>9.81</v>
@@ -517,26 +516,26 @@
       <c r="B4" s="1">
         <v>5.0121400000000003E-2</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4">
         <v>10.7</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4">
         <v>18.7</v>
       </c>
       <c r="E4" s="1">
         <v>1009</v>
       </c>
       <c r="F4" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G4" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H4" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I4" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J4" s="1">
         <v>9.81</v>
@@ -549,26 +548,26 @@
       <c r="B5" s="1">
         <v>2.0010099999999999E-2</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5">
         <v>10.7</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5">
         <v>16.3</v>
       </c>
       <c r="E5" s="1">
         <v>1009</v>
       </c>
       <c r="F5" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G5" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H5" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I5" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J5" s="1">
         <v>9.81</v>
@@ -581,26 +580,26 @@
       <c r="B6" s="1">
         <v>2.0010099999999999E-2</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6">
         <v>10.7</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6">
         <v>16</v>
       </c>
       <c r="E6" s="1">
         <v>1009</v>
       </c>
       <c r="F6" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G6" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H6" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I6" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J6" s="1">
         <v>9.81</v>
@@ -613,26 +612,26 @@
       <c r="B7" s="1">
         <v>2.0010099999999999E-2</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7">
         <v>10.7</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7">
         <v>15.6</v>
       </c>
       <c r="E7" s="1">
         <v>1009</v>
       </c>
       <c r="F7" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G7" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H7" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I7" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J7" s="1">
         <v>9.81</v>
@@ -645,26 +644,26 @@
       <c r="B8" s="1">
         <v>2.0010099999999999E-2</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8">
         <v>10.7</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8">
         <v>15.8</v>
       </c>
       <c r="E8" s="1">
         <v>1009</v>
       </c>
       <c r="F8" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G8" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H8" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I8" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J8" s="1">
         <v>9.81</v>
@@ -677,26 +676,26 @@
       <c r="B9" s="1">
         <v>0.10002469999999999</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9">
         <v>10.8</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9">
         <v>22.1</v>
       </c>
       <c r="E9" s="1">
         <v>1009</v>
       </c>
       <c r="F9" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G9" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H9" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I9" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J9" s="1">
         <v>9.81</v>
@@ -709,26 +708,26 @@
       <c r="B10" s="1">
         <v>0.10002469999999999</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10">
         <v>11.1</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10">
         <v>21.6</v>
       </c>
       <c r="E10" s="1">
         <v>1009</v>
       </c>
       <c r="F10" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G10" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H10" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I10" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J10" s="1">
         <v>9.81</v>
@@ -741,26 +740,26 @@
       <c r="B11" s="1">
         <v>0.10002469999999999</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11">
         <v>11.8</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11">
         <v>21.7</v>
       </c>
       <c r="E11" s="1">
         <v>1009</v>
       </c>
       <c r="F11" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G11" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H11" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I11" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J11" s="1">
         <v>9.81</v>
@@ -773,26 +772,26 @@
       <c r="B12" s="1">
         <v>0.10002469999999999</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12">
         <v>8.49</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12">
         <v>15.4</v>
       </c>
       <c r="E12" s="1">
         <v>1009</v>
       </c>
       <c r="F12" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G12" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H12" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I12" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J12" s="1">
         <v>9.81</v>
@@ -805,26 +804,26 @@
       <c r="B13" s="1">
         <v>0.10002469999999999</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13">
         <v>9.0399999999999991</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13">
         <v>17.399999999999999</v>
       </c>
       <c r="E13" s="1">
         <v>1009</v>
       </c>
       <c r="F13" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G13" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H13" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I13" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J13" s="1">
         <v>9.81</v>
@@ -837,26 +836,26 @@
       <c r="B14" s="1">
         <v>0.10002469999999999</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14">
         <v>9.4499999999999993</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14">
         <v>17.5</v>
       </c>
       <c r="E14" s="1">
         <v>1009</v>
       </c>
       <c r="F14" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G14" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H14" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I14" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J14" s="1">
         <v>9.81</v>
@@ -869,26 +868,26 @@
       <c r="B15" s="1">
         <v>5.0121400000000003E-2</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15">
         <v>9.1999999999999993</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15">
         <v>16</v>
       </c>
       <c r="E15" s="1">
         <v>1009</v>
       </c>
       <c r="F15" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G15" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H15" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I15" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J15" s="1">
         <v>9.81</v>
@@ -901,26 +900,26 @@
       <c r="B16" s="1">
         <v>5.0121400000000003E-2</v>
       </c>
-      <c r="C16" s="2">
+      <c r="C16">
         <v>9.32</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16">
         <v>15.6</v>
       </c>
       <c r="E16" s="1">
         <v>1009</v>
       </c>
       <c r="F16" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G16" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H16" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I16" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J16" s="1">
         <v>9.81</v>
@@ -933,26 +932,26 @@
       <c r="B17" s="1">
         <v>5.0121400000000003E-2</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17">
         <v>8.6300000000000008</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17">
         <v>14.8</v>
       </c>
       <c r="E17" s="1">
         <v>1009</v>
       </c>
       <c r="F17" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G17" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H17" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I17" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J17" s="1">
         <v>9.81</v>
@@ -965,26 +964,26 @@
       <c r="B18" s="1">
         <v>0.20006019999999999</v>
       </c>
-      <c r="C18" s="2">
+      <c r="C18">
         <v>9.4499999999999993</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18">
         <v>19.2</v>
       </c>
       <c r="E18" s="1">
         <v>1009</v>
       </c>
       <c r="F18" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G18" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H18" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I18" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J18" s="1">
         <v>9.81</v>
@@ -997,26 +996,26 @@
       <c r="B19" s="1">
         <v>0.20006019999999999</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19">
         <v>9.4499999999999993</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19">
         <v>19.7</v>
       </c>
       <c r="E19" s="1">
         <v>1009</v>
       </c>
       <c r="F19" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G19" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H19" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I19" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J19" s="1">
         <v>9.81</v>
@@ -1029,26 +1028,26 @@
       <c r="B20" s="1">
         <v>0.20006019999999999</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20">
         <v>10.1</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20">
         <v>20.3</v>
       </c>
       <c r="E20" s="1">
         <v>1009</v>
       </c>
       <c r="F20" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G20" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H20" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I20" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J20" s="1">
         <v>9.81</v>
@@ -1061,26 +1060,26 @@
       <c r="B21" s="1">
         <v>2.0010099999999999E-2</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21">
         <v>8.36</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21">
         <v>12.9</v>
       </c>
       <c r="E21" s="1">
         <v>1009</v>
       </c>
       <c r="F21" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G21" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H21" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I21" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J21" s="1">
         <v>9.81</v>
@@ -1093,26 +1092,26 @@
       <c r="B22" s="1">
         <v>2.0010099999999999E-2</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C22">
         <v>8.77</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22">
         <v>13.2</v>
       </c>
       <c r="E22" s="1">
         <v>1009</v>
       </c>
       <c r="F22" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G22" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H22" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I22" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J22" s="1">
         <v>9.81</v>
@@ -1125,26 +1124,26 @@
       <c r="B23" s="1">
         <v>2.0010099999999999E-2</v>
       </c>
-      <c r="C23" s="2">
+      <c r="C23">
         <v>10</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23">
         <v>14.3</v>
       </c>
       <c r="E23" s="1">
         <v>1009</v>
       </c>
       <c r="F23" s="1">
-        <v>15</v>
+        <v>12.164</v>
       </c>
       <c r="G23" s="1">
-        <v>90</v>
+        <v>15.3</v>
       </c>
       <c r="H23" s="1">
-        <v>0.4</v>
+        <v>0.42699999999999999</v>
       </c>
       <c r="I23" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J23" s="1">
         <v>9.81</v>

</xml_diff>

<commit_message>
2e serie mayo, jeudi
</commit_message>
<xml_diff>
--- a/Experiences/Mesures mayonnaise.xlsx
+++ b/Experiences/Mesures mayonnaise.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\Mines IC\TR Fluide\VS\Experiences\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10602154-A4DE-4D03-AF1B-36EDA3C5D8FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{528BE9FF-3B7E-419E-825F-FCB1B3096D50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{55767A0E-F7C5-4F3D-85D9-C64A23758580}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{55767A0E-F7C5-4F3D-85D9-C64A23758580}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>

</xml_diff>